<commit_message>
buscador integrado en el nav
</commit_message>
<xml_diff>
--- a/LISTAS/ma/REGATON DE GOMA DISMAY.xlsx
+++ b/LISTAS/ma/REGATON DE GOMA DISMAY.xlsx
@@ -736,14 +736,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="20" t="n">
-        <v>45182.62504073627</v>
+        <v>45219</v>
       </c>
       <c r="E1" s="3" t="n"/>
     </row>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5"/>
     <row r="6" ht="22.5" customHeight="1" s="16">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -789,21 +785,6 @@
       </c>
       <c r="E11" s="9" t="n"/>
     </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
     <row r="27" ht="18" customHeight="1" s="16">
       <c r="A27" s="10" t="inlineStr">
         <is>
@@ -835,7 +816,7 @@
       </c>
       <c r="C28" s="19" t="n"/>
       <c r="D28" s="5" t="n">
-        <v>5443.5</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1" s="16">
@@ -935,7 +916,6 @@
         </is>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
@@ -946,18 +926,18 @@
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="A35:D35"/>
     <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="A11:D11"/>
     <mergeCell ref="B27:C27"/>
-    <mergeCell ref="A9:D9"/>
     <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A35:D35"/>
     <mergeCell ref="A36:D36"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>